<commit_message>
Harden admin AI reports with DB rate limits and access control tests
</commit_message>
<xml_diff>
--- a/backend/US to API Mapping.xlsx
+++ b/backend/US to API Mapping.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\IITM BS Diploma\BSc LEVEL\SE\Merging Try 2\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5627377B-88DF-4A98-A14B-3EFB9D5D5B64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26D6BD67-1CCA-47B7-A4CF-7B745C2BC193}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{E373D3CA-1BFE-4B27-BD5E-FBAE2D0C403E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{E373D3CA-1BFE-4B27-BD5E-FBAE2D0C403E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="815" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1226" uniqueCount="323">
   <si>
     <t>EPIC 1 — User Authentication and Role Management</t>
   </si>
@@ -1011,7 +1012,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1039,6 +1040,17 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Fira Code"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1060,7 +1072,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1073,6 +1085,23 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4374,4 +4403,1755 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F761DEB-F9A6-4C28-8ABE-0441642A72EE}">
+  <dimension ref="A1:E112"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="3.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.88671875" style="6" customWidth="1"/>
+    <col min="3" max="3" width="57.77734375" style="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.44140625" style="10" customWidth="1"/>
+    <col min="5" max="5" width="39.21875" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.88671875" style="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B1" s="7" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="6">
+        <v>1</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="6">
+        <v>2</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="6">
+        <v>3</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="6">
+        <v>4</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="6">
+        <v>5</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="6">
+        <v>6</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="6">
+        <v>7</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="6">
+        <v>8</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="6">
+        <v>9</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="6">
+        <v>10</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="6">
+        <v>11</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="6">
+        <v>12</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="6">
+        <v>13</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="6">
+        <v>14</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="6">
+        <v>15</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="6">
+        <v>16</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A19" s="6">
+        <v>17</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="6">
+        <v>18</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="6">
+        <v>19</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="6">
+        <v>20</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="6">
+        <v>21</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B25" s="7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B26" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="D26" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="6">
+        <v>1</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="6">
+        <v>2</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A29" s="6">
+        <v>3</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="6">
+        <v>4</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="6">
+        <v>5</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="D31" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="6">
+        <v>6</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C32" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="D32" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A33" s="6">
+        <v>7</v>
+      </c>
+      <c r="B33" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="6">
+        <v>8</v>
+      </c>
+      <c r="B34" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C34" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="6">
+        <v>9</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="D35" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A36" s="6">
+        <v>10</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C36" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="D36" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="6">
+        <v>11</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="D37" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="6">
+        <v>12</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C38" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="D38" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A39" s="6">
+        <v>13</v>
+      </c>
+      <c r="B39" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C39" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="D39" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="6">
+        <v>14</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="C40" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D40" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E40" s="9" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="6">
+        <v>15</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="C41" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="D41" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="6">
+        <v>16</v>
+      </c>
+      <c r="B42" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="C42" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="D42" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="6">
+        <v>17</v>
+      </c>
+      <c r="B43" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="C43" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="D43" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E43" s="9" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="6">
+        <v>18</v>
+      </c>
+      <c r="B44" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="C44" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="D44" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E44" s="9" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="6">
+        <v>19</v>
+      </c>
+      <c r="B45" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="C45" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="D45" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E45" s="9" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="6">
+        <v>20</v>
+      </c>
+      <c r="B46" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="C46" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="D46" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E46" s="9" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A47" s="6">
+        <v>21</v>
+      </c>
+      <c r="B47" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="C47" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="D47" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="E47" s="9" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="6">
+        <v>22</v>
+      </c>
+      <c r="B48" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="C48" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="D48" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E48" s="9" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="6">
+        <v>23</v>
+      </c>
+      <c r="B49" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="C49" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="D49" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E49" s="9" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B51" s="7" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B52" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C52" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="D52" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="E52" s="8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="6">
+        <v>1</v>
+      </c>
+      <c r="B53" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="C53" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="D53" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E53" s="9" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="6">
+        <v>2</v>
+      </c>
+      <c r="B54" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="C54" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="D54" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="E54" s="9" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A55" s="6">
+        <v>3</v>
+      </c>
+      <c r="B55" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="C55" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="D55" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="E55" s="9" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="6">
+        <v>4</v>
+      </c>
+      <c r="B56" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="C56" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="D56" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E56" s="9" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" s="6">
+        <v>5</v>
+      </c>
+      <c r="B57" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="C57" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="D57" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E57" s="9" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" s="6">
+        <v>6</v>
+      </c>
+      <c r="B58" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="C58" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="D58" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E58" s="9" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="6">
+        <v>7</v>
+      </c>
+      <c r="B59" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="C59" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="D59" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E59" s="9" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" s="6">
+        <v>8</v>
+      </c>
+      <c r="B60" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="C60" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="D60" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="E60" s="9" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A61" s="6">
+        <v>9</v>
+      </c>
+      <c r="B61" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="C61" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="D61" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="E61" s="9" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" s="6">
+        <v>10</v>
+      </c>
+      <c r="B62" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="C62" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="D62" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E62" s="9" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" s="6">
+        <v>11</v>
+      </c>
+      <c r="B63" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="C63" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="D63" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E63" s="9" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="6">
+        <v>12</v>
+      </c>
+      <c r="B64" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="C64" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="D64" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E64" s="9" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="6">
+        <v>13</v>
+      </c>
+      <c r="B65" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="C65" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="D65" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E65" s="9" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" s="6">
+        <v>14</v>
+      </c>
+      <c r="B66" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="C66" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="D66" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E66" s="9" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" s="6">
+        <v>15</v>
+      </c>
+      <c r="B67" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="C67" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="D67" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E67" s="9" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="6">
+        <v>16</v>
+      </c>
+      <c r="B68" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="C68" s="12" t="s">
+        <v>192</v>
+      </c>
+      <c r="D68" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E68" s="9" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" s="6">
+        <v>17</v>
+      </c>
+      <c r="B69" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="C69" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="D69" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E69" s="9" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B71" s="7" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B72" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C72" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="D72" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="E72" s="8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" s="6">
+        <v>1</v>
+      </c>
+      <c r="B73" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="C73" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="D73" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E73" s="9" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="6">
+        <v>2</v>
+      </c>
+      <c r="B74" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="C74" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="D74" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E74" s="9" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="6">
+        <v>3</v>
+      </c>
+      <c r="B75" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="C75" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="D75" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E75" s="9" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" s="6">
+        <v>4</v>
+      </c>
+      <c r="B76" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="C76" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="D76" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E76" s="9" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="6">
+        <v>5</v>
+      </c>
+      <c r="B77" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="C77" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="D77" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E77" s="9" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B79" s="7" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B80" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C80" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="D80" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="E80" s="8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="6">
+        <v>1</v>
+      </c>
+      <c r="B81" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="C81" s="12" t="s">
+        <v>225</v>
+      </c>
+      <c r="D81" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E81" s="9" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="6">
+        <v>2</v>
+      </c>
+      <c r="B82" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="C82" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="D82" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E82" s="9" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="6">
+        <v>3</v>
+      </c>
+      <c r="B83" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="C83" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="D83" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E83" s="9" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A84" s="6">
+        <v>4</v>
+      </c>
+      <c r="B84" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="C84" s="12" t="s">
+        <v>234</v>
+      </c>
+      <c r="D84" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E84" s="9" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A85" s="6">
+        <v>5</v>
+      </c>
+      <c r="B85" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="C85" s="12" t="s">
+        <v>237</v>
+      </c>
+      <c r="D85" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E85" s="9" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A86" s="6">
+        <v>6</v>
+      </c>
+      <c r="B86" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="C86" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="D86" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E86" s="9" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A87" s="6">
+        <v>7</v>
+      </c>
+      <c r="B87" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="C87" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="D87" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E87" s="9" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A88" s="6">
+        <v>8</v>
+      </c>
+      <c r="B88" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="C88" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="D88" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E88" s="9" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A89" s="6">
+        <v>9</v>
+      </c>
+      <c r="B89" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C89" s="12" t="s">
+        <v>252</v>
+      </c>
+      <c r="D89" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E89" s="9" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A90" s="6">
+        <v>10</v>
+      </c>
+      <c r="B90" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C90" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="D90" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E90" s="9" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" s="6">
+        <v>11</v>
+      </c>
+      <c r="B91" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C91" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="D91" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E91" s="9" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" s="6">
+        <v>12</v>
+      </c>
+      <c r="B92" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C92" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="D92" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E92" s="9" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A93" s="6">
+        <v>13</v>
+      </c>
+      <c r="B93" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C93" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="D93" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E93" s="9" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A94" s="6">
+        <v>14</v>
+      </c>
+      <c r="B94" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C94" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="D94" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E94" s="9" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A95" s="6">
+        <v>15</v>
+      </c>
+      <c r="B95" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C95" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="D95" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E95" s="9" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A96" s="6">
+        <v>16</v>
+      </c>
+      <c r="B96" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C96" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="D96" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="E96" s="9" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A97" s="6">
+        <v>17</v>
+      </c>
+      <c r="B97" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C97" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="D97" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E97" s="9" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A98" s="6">
+        <v>18</v>
+      </c>
+      <c r="B98" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C98" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="D98" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E98" s="9" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A99" s="6">
+        <v>19</v>
+      </c>
+      <c r="B99" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C99" s="12" t="s">
+        <v>281</v>
+      </c>
+      <c r="D99" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E99" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" s="6">
+        <v>20</v>
+      </c>
+      <c r="B100" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C100" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="D100" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E100" s="9" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A101" s="6">
+        <v>21</v>
+      </c>
+      <c r="B101" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C101" s="12" t="s">
+        <v>287</v>
+      </c>
+      <c r="D101" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E101" s="9" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" s="6">
+        <v>22</v>
+      </c>
+      <c r="B102" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C102" s="12" t="s">
+        <v>290</v>
+      </c>
+      <c r="D102" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E102" s="9" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" s="6">
+        <v>23</v>
+      </c>
+      <c r="B103" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C103" s="12" t="s">
+        <v>294</v>
+      </c>
+      <c r="D103" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E103" s="9" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" s="6">
+        <v>24</v>
+      </c>
+      <c r="B104" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C104" s="12" t="s">
+        <v>297</v>
+      </c>
+      <c r="D104" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E104" s="9" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B106" s="7" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B107" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C107" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="D107" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="E107" s="8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A108" s="6">
+        <v>1</v>
+      </c>
+      <c r="B108" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="C108" s="12" t="s">
+        <v>305</v>
+      </c>
+      <c r="D108" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E108" s="9" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A109" s="6">
+        <v>2</v>
+      </c>
+      <c r="B109" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="C109" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="D109" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E109" s="9" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A110" s="6">
+        <v>3</v>
+      </c>
+      <c r="B110" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="C110" s="12" t="s">
+        <v>311</v>
+      </c>
+      <c r="D110" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="E110" s="9" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A111" s="6">
+        <v>4</v>
+      </c>
+      <c r="B111" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="C111" s="12" t="s">
+        <v>314</v>
+      </c>
+      <c r="D111" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="E111" s="9" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A112" s="6">
+        <v>5</v>
+      </c>
+      <c r="B112" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="C112" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="D112" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E112" s="9" t="s">
+        <v>319</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>